<commit_message>
feat: PSW graduate tax contribution - Jupyter notebook with real payslip data
</commit_message>
<xml_diff>
--- a/UK_Immigration_Tax_Fairness.xlsx
+++ b/UK_Immigration_Tax_Fairness.xlsx
@@ -956,7 +956,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NHS (1 A&amp;E visit — paid for own medicine)</t>
+          <t>NHS (1 A&amp;E visit â€” paid for own medicine)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>£42,140</t>
+          <t>Â£42,140</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>£5,793</t>
+          <t>Â£5,793</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>£4,491</t>
+          <t>Â£4,491</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>£30,065</t>
+          <t>Â£30,065</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>£150</t>
+          <t>Â£150</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>£29,915</t>
+          <t>Â£29,915</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>£2,480</t>
+          <t>Â£2,480</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>£4,609</t>
+          <t>Â£4,609</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>£150</t>
+          <t>Â£150</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: PSW graduate tax contribution - real payslip data, NHS reference costs
</commit_message>
<xml_diff>
--- a/UK_Immigration_Tax_Fairness.xlsx
+++ b/UK_Immigration_Tax_Fairness.xlsx
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>£150</t>
+          <t>£96</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>£29,915</t>
+          <t>£29,969</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>£150</t>
+          <t>£96</t>
         </is>
       </c>
     </row>

</xml_diff>